<commit_message>
Mise à jour des fichiers de mapping
</commit_message>
<xml_diff>
--- a/data/mappings/Mapp_tab.xlsx
+++ b/data/mappings/Mapp_tab.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7522BE1D-35E4-470D-B075-50D339920401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$D$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$B$1:$B$33</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
   <si>
     <t>Membres - Niveau 2</t>
   </si>
@@ -180,7 +181,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -242,40 +243,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -557,8 +562,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D33"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="38.36328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.54296875" style="1" customWidth="1"/>
@@ -1030,7 +1035,22 @@
         <v>786443908</v>
       </c>
     </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="4">
+        <v>504</v>
+      </c>
+      <c r="D34" s="12">
+        <v>786451920</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="B1:B33" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>